<commit_message>
chore: update monthly dashboard
</commit_message>
<xml_diff>
--- a/downloads/勞動基金月度揭露_可持續更新.xlsx
+++ b/downloads/勞動基金月度揭露_可持續更新.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1650" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1670" uniqueCount="187">
   <si>
     <t>勞動基金運用局｜四大基金月度儀表板</t>
   </si>
@@ -73,31 +73,31 @@
     <t>國外投資</t>
   </si>
   <si>
-    <t>自行運用-固定收益</t>
-  </si>
-  <si>
-    <t>自行運用-權益證券</t>
-  </si>
-  <si>
-    <t>自行運用-另類投資</t>
+    <t>自行運用-國外-固定收益</t>
+  </si>
+  <si>
+    <t>自行運用-國外-權益證券</t>
+  </si>
+  <si>
+    <t>自行運用-國外-另類投資</t>
   </si>
   <si>
     <t>委託經營</t>
   </si>
   <si>
-    <t>國內委託經營</t>
+    <t>委託經營-國內-權益證券</t>
   </si>
   <si>
     <t>國外委託經營</t>
   </si>
   <si>
-    <t>委託經營-固定收益</t>
-  </si>
-  <si>
-    <t>委託經營-權益證券</t>
-  </si>
-  <si>
-    <t>委託經營-另類投資</t>
+    <t>委託經營-國外-固定收益</t>
+  </si>
+  <si>
+    <t>委託經營-國外-權益證券</t>
+  </si>
+  <si>
+    <t>委託經營-國外-另類投資</t>
   </si>
   <si>
     <t>合計</t>
@@ -292,6 +292,9 @@
     <t>106年第一次委託經營(續約)</t>
   </si>
   <si>
+    <t>新增</t>
+  </si>
+  <si>
     <t>解約</t>
   </si>
   <si>
@@ -334,9 +337,6 @@
     <t>100-1全球基本面指數被動股票型（續約3）</t>
   </si>
   <si>
-    <t>新增</t>
-  </si>
-  <si>
     <t>100-1全球不動產有價證券型（續約2）</t>
   </si>
   <si>
@@ -439,7 +439,7 @@
     <t>CBRE</t>
   </si>
   <si>
-    <t>Clearbridge</t>
+    <t>ClearBridge</t>
   </si>
   <si>
     <t>110-1全球多元資產型</t>
@@ -533,9 +533,6 @@
   </si>
   <si>
     <t>107-1絕對報酬股票型(續約)</t>
-  </si>
-  <si>
-    <t>ClearBridge</t>
   </si>
   <si>
     <t>100年全球主動股票型(續約2)</t>
@@ -1721,7 +1718,7 @@
         <v>7</v>
       </c>
       <c r="B47" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C47" s="1">
         <v>68461127545</v>
@@ -1987,7 +1984,7 @@
         <v>8</v>
       </c>
       <c r="B66" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C66" s="1">
         <v>100575817739</v>
@@ -2116,7 +2113,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J110"/>
+  <dimension ref="A1:J114"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="22" customWidth="1"/>
@@ -5158,122 +5155,122 @@
     </row>
     <row r="102" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B102" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="C102" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="D102" s="1">
-        <v>3000000000</v>
+        <v>500000000</v>
       </c>
       <c r="E102" s="1">
-        <v>3958912304</v>
+        <v>1165423958</v>
       </c>
       <c r="F102" s="7">
-        <v>1380163332</v>
+        <v>1165423958</v>
       </c>
       <c r="G102" t="s">
-        <v>44</v>
+        <v>92</v>
       </c>
       <c r="H102" t="s">
         <v>45</v>
       </c>
       <c r="I102" s="5"/>
       <c r="J102" s="5">
-        <v>1.1673</v>
+        <v>1.2554</v>
       </c>
     </row>
     <row r="103" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B103" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="C103" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="D103" s="1">
-        <v>3000000000</v>
+        <v>500000000</v>
       </c>
       <c r="E103" s="1">
-        <v>3975895368</v>
+        <v>1151125436</v>
       </c>
       <c r="F103" s="7">
-        <v>1397858568</v>
+        <v>1151125436</v>
       </c>
       <c r="G103" t="s">
-        <v>44</v>
+        <v>92</v>
       </c>
       <c r="H103" t="s">
         <v>45</v>
       </c>
       <c r="I103" s="5"/>
       <c r="J103" s="5">
-        <v>1.1673</v>
+        <v>1.2554</v>
       </c>
     </row>
     <row r="104" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B104" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="C104" t="s">
-        <v>81</v>
+        <v>43</v>
       </c>
       <c r="D104" s="1">
-        <v>400000000</v>
+        <v>500000000</v>
       </c>
       <c r="E104" s="1">
-        <v>381187393</v>
+        <v>1148829895</v>
       </c>
       <c r="F104" s="7">
-        <v>-30591888</v>
+        <v>1148829895</v>
       </c>
       <c r="G104" t="s">
-        <v>44</v>
+        <v>92</v>
       </c>
       <c r="H104" t="s">
         <v>45</v>
       </c>
       <c r="I104" s="5"/>
       <c r="J104" s="5">
-        <v>0.009000000000000001</v>
+        <v>1.2554</v>
       </c>
     </row>
     <row r="105" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B105" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="C105" t="s">
-        <v>66</v>
+        <v>50</v>
       </c>
       <c r="D105" s="1">
-        <v>400000000</v>
+        <v>500000000</v>
       </c>
       <c r="E105" s="1">
-        <v>333326095</v>
+        <v>1186966069</v>
       </c>
       <c r="F105" s="7">
-        <v>-59815011</v>
+        <v>1186966069</v>
       </c>
       <c r="G105" t="s">
-        <v>44</v>
+        <v>92</v>
       </c>
       <c r="H105" t="s">
         <v>45</v>
       </c>
       <c r="I105" s="5"/>
       <c r="J105" s="5">
-        <v>0.009000000000000001</v>
+        <v>1.2554</v>
       </c>
     </row>
     <row r="106" spans="1:10" x14ac:dyDescent="0.25">
@@ -5281,19 +5278,19 @@
         <v>8</v>
       </c>
       <c r="B106" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="C106" t="s">
-        <v>43</v>
+        <v>66</v>
       </c>
       <c r="D106" s="1">
-        <v>400000000</v>
+        <v>3000000000</v>
       </c>
       <c r="E106" s="1">
-        <v>341538111</v>
+        <v>3958912304</v>
       </c>
       <c r="F106" s="7">
-        <v>-55332604</v>
+        <v>1380163332</v>
       </c>
       <c r="G106" t="s">
         <v>44</v>
@@ -5303,120 +5300,240 @@
       </c>
       <c r="I106" s="5"/>
       <c r="J106" s="5">
-        <v>0.009000000000000001</v>
+        <v>1.1673</v>
       </c>
     </row>
     <row r="107" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B107" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="C107" t="s">
-        <v>60</v>
+        <v>43</v>
       </c>
       <c r="D107" s="1">
-        <v>0</v>
+        <v>3000000000</v>
       </c>
       <c r="E107" s="1">
-        <v>0</v>
+        <v>3975895368</v>
       </c>
       <c r="F107" s="7">
-        <v>-1528889549</v>
+        <v>1397858568</v>
       </c>
       <c r="G107" t="s">
-        <v>92</v>
+        <v>44</v>
       </c>
       <c r="H107" t="s">
         <v>45</v>
       </c>
       <c r="I107" s="5"/>
-      <c r="J107" s="5"/>
+      <c r="J107" s="5">
+        <v>1.1673</v>
+      </c>
     </row>
     <row r="108" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B108" t="s">
         <v>80</v>
       </c>
       <c r="C108" t="s">
-        <v>66</v>
+        <v>81</v>
       </c>
       <c r="D108" s="1">
-        <v>0</v>
+        <v>400000000</v>
       </c>
       <c r="E108" s="1">
-        <v>0</v>
+        <v>381187393</v>
       </c>
       <c r="F108" s="7">
-        <v>-1474347055</v>
+        <v>-30591888</v>
       </c>
       <c r="G108" t="s">
-        <v>92</v>
+        <v>44</v>
       </c>
       <c r="H108" t="s">
         <v>45</v>
       </c>
       <c r="I108" s="5"/>
-      <c r="J108" s="5"/>
+      <c r="J108" s="5">
+        <v>0.009000000000000001</v>
+      </c>
     </row>
     <row r="109" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B109" t="s">
         <v>80</v>
       </c>
       <c r="C109" t="s">
-        <v>43</v>
+        <v>66</v>
       </c>
       <c r="D109" s="1">
-        <v>0</v>
+        <v>400000000</v>
       </c>
       <c r="E109" s="1">
-        <v>0</v>
+        <v>333326095</v>
       </c>
       <c r="F109" s="7">
-        <v>-1489331693</v>
+        <v>-59815011</v>
       </c>
       <c r="G109" t="s">
-        <v>92</v>
+        <v>44</v>
       </c>
       <c r="H109" t="s">
         <v>45</v>
       </c>
       <c r="I109" s="5"/>
-      <c r="J109" s="5"/>
+      <c r="J109" s="5">
+        <v>0.009000000000000001</v>
+      </c>
     </row>
     <row r="110" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B110" t="s">
         <v>80</v>
       </c>
       <c r="C110" t="s">
+        <v>43</v>
+      </c>
+      <c r="D110" s="1">
+        <v>400000000</v>
+      </c>
+      <c r="E110" s="1">
+        <v>341538111</v>
+      </c>
+      <c r="F110" s="7">
+        <v>-55332604</v>
+      </c>
+      <c r="G110" t="s">
+        <v>44</v>
+      </c>
+      <c r="H110" t="s">
+        <v>45</v>
+      </c>
+      <c r="I110" s="5"/>
+      <c r="J110" s="5">
+        <v>0.009000000000000001</v>
+      </c>
+    </row>
+    <row r="111" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>5</v>
+      </c>
+      <c r="B111" t="s">
+        <v>80</v>
+      </c>
+      <c r="C111" t="s">
+        <v>60</v>
+      </c>
+      <c r="D111" s="1">
+        <v>0</v>
+      </c>
+      <c r="E111" s="1">
+        <v>0</v>
+      </c>
+      <c r="F111" s="7">
+        <v>-1528889549</v>
+      </c>
+      <c r="G111" t="s">
+        <v>93</v>
+      </c>
+      <c r="H111" t="s">
+        <v>45</v>
+      </c>
+      <c r="I111" s="5"/>
+      <c r="J111" s="5"/>
+    </row>
+    <row r="112" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>5</v>
+      </c>
+      <c r="B112" t="s">
+        <v>80</v>
+      </c>
+      <c r="C112" t="s">
+        <v>66</v>
+      </c>
+      <c r="D112" s="1">
+        <v>0</v>
+      </c>
+      <c r="E112" s="1">
+        <v>0</v>
+      </c>
+      <c r="F112" s="7">
+        <v>-1474347055</v>
+      </c>
+      <c r="G112" t="s">
+        <v>93</v>
+      </c>
+      <c r="H112" t="s">
+        <v>45</v>
+      </c>
+      <c r="I112" s="5"/>
+      <c r="J112" s="5"/>
+    </row>
+    <row r="113" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>5</v>
+      </c>
+      <c r="B113" t="s">
+        <v>80</v>
+      </c>
+      <c r="C113" t="s">
+        <v>43</v>
+      </c>
+      <c r="D113" s="1">
+        <v>0</v>
+      </c>
+      <c r="E113" s="1">
+        <v>0</v>
+      </c>
+      <c r="F113" s="7">
+        <v>-1489331693</v>
+      </c>
+      <c r="G113" t="s">
+        <v>93</v>
+      </c>
+      <c r="H113" t="s">
+        <v>45</v>
+      </c>
+      <c r="I113" s="5"/>
+      <c r="J113" s="5"/>
+    </row>
+    <row r="114" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>5</v>
+      </c>
+      <c r="B114" t="s">
+        <v>80</v>
+      </c>
+      <c r="C114" t="s">
         <v>77</v>
       </c>
-      <c r="D110" s="1">
+      <c r="D114" s="1">
         <v>0</v>
       </c>
-      <c r="E110" s="1">
+      <c r="E114" s="1">
         <v>0</v>
       </c>
-      <c r="F110" s="7">
+      <c r="F114" s="7">
         <v>-1492945981</v>
       </c>
-      <c r="G110" t="s">
-        <v>92</v>
-      </c>
-      <c r="H110" t="s">
-        <v>45</v>
-      </c>
-      <c r="I110" s="5"/>
-      <c r="J110" s="5"/>
+      <c r="G114" t="s">
+        <v>93</v>
+      </c>
+      <c r="H114" t="s">
+        <v>45</v>
+      </c>
+      <c r="I114" s="5"/>
+      <c r="J114" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5473,10 +5590,10 @@
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D2" s="1">
         <v>900495639</v>
@@ -5491,7 +5608,7 @@
         <v>44</v>
       </c>
       <c r="H2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I2" s="5"/>
       <c r="J2" s="5">
@@ -5503,10 +5620,10 @@
         <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D3" s="1">
         <v>1338657958</v>
@@ -5521,7 +5638,7 @@
         <v>44</v>
       </c>
       <c r="H3" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I3" s="5"/>
       <c r="J3" s="5">
@@ -5533,10 +5650,10 @@
         <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C4" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D4" s="1">
         <v>2408967886</v>
@@ -5551,7 +5668,7 @@
         <v>44</v>
       </c>
       <c r="H4" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I4" s="5"/>
       <c r="J4" s="5">
@@ -5563,7 +5680,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C5" t="s">
         <v>79</v>
@@ -5581,7 +5698,7 @@
         <v>44</v>
       </c>
       <c r="H5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I5" s="5"/>
       <c r="J5" s="5">
@@ -5593,10 +5710,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D6" s="1">
         <v>1585120883</v>
@@ -5611,7 +5728,7 @@
         <v>44</v>
       </c>
       <c r="H6" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I6" s="5"/>
       <c r="J6" s="5">
@@ -5623,10 +5740,10 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D7" s="1">
         <v>656507639</v>
@@ -5641,7 +5758,7 @@
         <v>44</v>
       </c>
       <c r="H7" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I7" s="5"/>
       <c r="J7" s="5">
@@ -5653,7 +5770,7 @@
         <v>5</v>
       </c>
       <c r="B8" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C8" t="s">
         <v>79</v>
@@ -5671,7 +5788,7 @@
         <v>44</v>
       </c>
       <c r="H8" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I8" s="5"/>
       <c r="J8" s="5">
@@ -5683,10 +5800,10 @@
         <v>5</v>
       </c>
       <c r="B9" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C9" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D9" s="1">
         <v>1783655177</v>
@@ -5701,7 +5818,7 @@
         <v>44</v>
       </c>
       <c r="H9" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I9" s="5"/>
       <c r="J9" s="5">
@@ -5713,10 +5830,10 @@
         <v>5</v>
       </c>
       <c r="B10" t="s">
+        <v>106</v>
+      </c>
+      <c r="C10" t="s">
         <v>105</v>
-      </c>
-      <c r="C10" t="s">
-        <v>104</v>
       </c>
       <c r="D10" s="1">
         <v>1683240295</v>
@@ -5728,10 +5845,10 @@
         <v>1714089252</v>
       </c>
       <c r="G10" t="s">
-        <v>106</v>
+        <v>92</v>
       </c>
       <c r="H10" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I10" s="5"/>
       <c r="J10" s="5">
@@ -5743,7 +5860,7 @@
         <v>5</v>
       </c>
       <c r="B11" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C11" t="s">
         <v>79</v>
@@ -5758,10 +5875,10 @@
         <v>1711777799</v>
       </c>
       <c r="G11" t="s">
-        <v>106</v>
+        <v>92</v>
       </c>
       <c r="H11" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I11" s="5"/>
       <c r="J11" s="5">
@@ -5791,7 +5908,7 @@
         <v>44</v>
       </c>
       <c r="H12" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I12" s="5"/>
       <c r="J12" s="5"/>
@@ -5804,7 +5921,7 @@
         <v>107</v>
       </c>
       <c r="C13" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D13" s="1">
         <v>1417127452</v>
@@ -5819,7 +5936,7 @@
         <v>44</v>
       </c>
       <c r="H13" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I13" s="5"/>
       <c r="J13" s="5"/>
@@ -5847,7 +5964,7 @@
         <v>44</v>
       </c>
       <c r="H14" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I14" s="5"/>
       <c r="J14" s="5">
@@ -5862,7 +5979,7 @@
         <v>111</v>
       </c>
       <c r="C15" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D15" s="1">
         <v>1263392347</v>
@@ -5877,7 +5994,7 @@
         <v>44</v>
       </c>
       <c r="H15" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I15" s="5"/>
       <c r="J15" s="5">
@@ -5907,7 +6024,7 @@
         <v>44</v>
       </c>
       <c r="H16" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I16" s="5"/>
       <c r="J16" s="5">
@@ -5937,7 +6054,7 @@
         <v>44</v>
       </c>
       <c r="H17" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I17" s="5"/>
       <c r="J17" s="5">
@@ -5967,7 +6084,7 @@
         <v>44</v>
       </c>
       <c r="H18" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I18" s="5"/>
       <c r="J18" s="5">
@@ -5997,7 +6114,7 @@
         <v>44</v>
       </c>
       <c r="H19" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I19" s="5"/>
       <c r="J19" s="5">
@@ -6027,7 +6144,7 @@
         <v>44</v>
       </c>
       <c r="H20" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I20" s="5"/>
       <c r="J20" s="5">
@@ -6057,7 +6174,7 @@
         <v>44</v>
       </c>
       <c r="H21" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I21" s="5"/>
       <c r="J21" s="5">
@@ -6087,7 +6204,7 @@
         <v>44</v>
       </c>
       <c r="H22" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I22" s="5"/>
       <c r="J22" s="5">
@@ -6117,7 +6234,7 @@
         <v>44</v>
       </c>
       <c r="H23" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I23" s="5"/>
       <c r="J23" s="5">
@@ -6144,10 +6261,10 @@
         <v>3866001108</v>
       </c>
       <c r="G24" t="s">
-        <v>106</v>
+        <v>92</v>
       </c>
       <c r="H24" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I24" s="5"/>
       <c r="J24" s="5">
@@ -6177,7 +6294,7 @@
         <v>44</v>
       </c>
       <c r="H25" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I25" s="5"/>
       <c r="J25" s="5">
@@ -6204,10 +6321,10 @@
         <v>1318692011</v>
       </c>
       <c r="G26" t="s">
-        <v>106</v>
+        <v>92</v>
       </c>
       <c r="H26" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I26" s="5"/>
       <c r="J26" s="5">
@@ -6234,10 +6351,10 @@
         <v>1836404740</v>
       </c>
       <c r="G27" t="s">
-        <v>106</v>
+        <v>92</v>
       </c>
       <c r="H27" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I27" s="5"/>
       <c r="J27" s="5">
@@ -6267,7 +6384,7 @@
         <v>44</v>
       </c>
       <c r="H28" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I28" s="5"/>
       <c r="J28" s="5">
@@ -6297,7 +6414,7 @@
         <v>44</v>
       </c>
       <c r="H29" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I29" s="5"/>
       <c r="J29" s="5">
@@ -6327,7 +6444,7 @@
         <v>44</v>
       </c>
       <c r="H30" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I30" s="5"/>
       <c r="J30" s="5">
@@ -6342,7 +6459,7 @@
         <v>127</v>
       </c>
       <c r="C31" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D31" s="1">
         <v>849045562</v>
@@ -6357,7 +6474,7 @@
         <v>44</v>
       </c>
       <c r="H31" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I31" s="5"/>
       <c r="J31" s="5">
@@ -6387,7 +6504,7 @@
         <v>44</v>
       </c>
       <c r="H32" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I32" s="5"/>
       <c r="J32" s="5">
@@ -6417,7 +6534,7 @@
         <v>44</v>
       </c>
       <c r="H33" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I33" s="5"/>
       <c r="J33" s="5"/>
@@ -6445,7 +6562,7 @@
         <v>44</v>
       </c>
       <c r="H34" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I34" s="5"/>
       <c r="J34" s="5"/>
@@ -6473,7 +6590,7 @@
         <v>44</v>
       </c>
       <c r="H35" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I35" s="5"/>
       <c r="J35" s="5"/>
@@ -6486,7 +6603,7 @@
         <v>133</v>
       </c>
       <c r="C36" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D36" s="1">
         <v>1006698949</v>
@@ -6501,7 +6618,7 @@
         <v>44</v>
       </c>
       <c r="H36" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I36" s="5"/>
       <c r="J36" s="5">
@@ -6531,7 +6648,7 @@
         <v>44</v>
       </c>
       <c r="H37" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I37" s="5"/>
       <c r="J37" s="5">
@@ -6561,7 +6678,7 @@
         <v>44</v>
       </c>
       <c r="H38" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I38" s="5"/>
       <c r="J38" s="5">
@@ -6576,7 +6693,7 @@
         <v>133</v>
       </c>
       <c r="C39" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D39" s="1">
         <v>806462703</v>
@@ -6591,7 +6708,7 @@
         <v>44</v>
       </c>
       <c r="H39" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I39" s="5"/>
       <c r="J39" s="5">
@@ -6621,7 +6738,7 @@
         <v>44</v>
       </c>
       <c r="H40" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I40" s="5"/>
       <c r="J40" s="5">
@@ -6651,7 +6768,7 @@
         <v>44</v>
       </c>
       <c r="H41" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I41" s="5"/>
       <c r="J41" s="5">
@@ -6666,7 +6783,7 @@
         <v>133</v>
       </c>
       <c r="C42" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D42" s="1">
         <v>441937598</v>
@@ -6681,7 +6798,7 @@
         <v>44</v>
       </c>
       <c r="H42" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I42" s="5"/>
       <c r="J42" s="5">
@@ -6711,7 +6828,7 @@
         <v>44</v>
       </c>
       <c r="H43" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I43" s="5"/>
       <c r="J43" s="5">
@@ -6726,7 +6843,7 @@
         <v>137</v>
       </c>
       <c r="C44" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D44" s="1">
         <v>558802476</v>
@@ -6741,7 +6858,7 @@
         <v>44</v>
       </c>
       <c r="H44" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I44" s="5"/>
       <c r="J44" s="5">
@@ -6756,7 +6873,7 @@
         <v>137</v>
       </c>
       <c r="C45" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D45" s="1">
         <v>674765647</v>
@@ -6771,7 +6888,7 @@
         <v>44</v>
       </c>
       <c r="H45" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I45" s="5"/>
       <c r="J45" s="5">
@@ -6801,7 +6918,7 @@
         <v>44</v>
       </c>
       <c r="H46" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I46" s="5"/>
       <c r="J46" s="5">
@@ -6831,7 +6948,7 @@
         <v>44</v>
       </c>
       <c r="H47" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I47" s="5"/>
       <c r="J47" s="5">
@@ -6861,7 +6978,7 @@
         <v>44</v>
       </c>
       <c r="H48" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I48" s="5"/>
       <c r="J48" s="5">
@@ -6891,7 +7008,7 @@
         <v>44</v>
       </c>
       <c r="H49" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I49" s="5"/>
       <c r="J49" s="5">
@@ -6921,7 +7038,7 @@
         <v>44</v>
       </c>
       <c r="H50" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I50" s="5"/>
       <c r="J50" s="5"/>
@@ -6934,7 +7051,7 @@
         <v>142</v>
       </c>
       <c r="C51" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D51" s="1">
         <v>400000000</v>
@@ -6949,7 +7066,7 @@
         <v>44</v>
       </c>
       <c r="H51" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I51" s="5"/>
       <c r="J51" s="5"/>
@@ -6977,7 +7094,7 @@
         <v>44</v>
       </c>
       <c r="H52" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I52" s="5"/>
       <c r="J52" s="5"/>
@@ -7005,7 +7122,7 @@
         <v>44</v>
       </c>
       <c r="H53" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I53" s="5"/>
       <c r="J53" s="5"/>
@@ -7033,7 +7150,7 @@
         <v>44</v>
       </c>
       <c r="H54" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I54" s="5"/>
       <c r="J54" s="5"/>
@@ -7061,7 +7178,7 @@
         <v>44</v>
       </c>
       <c r="H55" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I55" s="5"/>
       <c r="J55" s="5"/>
@@ -7089,7 +7206,7 @@
         <v>44</v>
       </c>
       <c r="H56" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I56" s="5"/>
       <c r="J56" s="5"/>
@@ -7117,7 +7234,7 @@
         <v>44</v>
       </c>
       <c r="H57" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I57" s="5"/>
       <c r="J57" s="5"/>
@@ -7145,7 +7262,7 @@
         <v>44</v>
       </c>
       <c r="H58" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I58" s="5"/>
       <c r="J58" s="5"/>
@@ -7173,7 +7290,7 @@
         <v>44</v>
       </c>
       <c r="H59" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I59" s="5"/>
       <c r="J59" s="5"/>
@@ -7201,7 +7318,7 @@
         <v>44</v>
       </c>
       <c r="H60" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I60" s="5"/>
       <c r="J60" s="5"/>
@@ -7229,7 +7346,7 @@
         <v>44</v>
       </c>
       <c r="H61" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I61" s="5"/>
       <c r="J61" s="5"/>
@@ -7242,7 +7359,7 @@
         <v>149</v>
       </c>
       <c r="C62" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D62" s="1">
         <v>500000000</v>
@@ -7257,7 +7374,7 @@
         <v>44</v>
       </c>
       <c r="H62" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I62" s="5"/>
       <c r="J62" s="5"/>
@@ -7285,7 +7402,7 @@
         <v>44</v>
       </c>
       <c r="H63" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I63" s="5"/>
       <c r="J63" s="5"/>
@@ -7313,7 +7430,7 @@
         <v>44</v>
       </c>
       <c r="H64" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I64" s="5"/>
       <c r="J64" s="5"/>
@@ -7341,7 +7458,7 @@
         <v>44</v>
       </c>
       <c r="H65" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I65" s="5"/>
       <c r="J65" s="5"/>
@@ -7369,7 +7486,7 @@
         <v>44</v>
       </c>
       <c r="H66" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I66" s="5"/>
       <c r="J66" s="5">
@@ -7396,10 +7513,10 @@
         <v>544159304</v>
       </c>
       <c r="G67" t="s">
-        <v>106</v>
+        <v>92</v>
       </c>
       <c r="H67" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I67" s="5"/>
       <c r="J67" s="5">
@@ -7414,7 +7531,7 @@
         <v>151</v>
       </c>
       <c r="C68" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D68" s="1">
         <v>400000000</v>
@@ -7429,7 +7546,7 @@
         <v>44</v>
       </c>
       <c r="H68" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I68" s="5"/>
       <c r="J68" s="5">
@@ -7459,7 +7576,7 @@
         <v>44</v>
       </c>
       <c r="H69" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I69" s="5"/>
       <c r="J69" s="5">
@@ -7489,7 +7606,7 @@
         <v>44</v>
       </c>
       <c r="H70" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I70" s="5"/>
       <c r="J70" s="5">
@@ -7519,7 +7636,7 @@
         <v>44</v>
       </c>
       <c r="H71" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I71" s="5"/>
       <c r="J71" s="5">
@@ -7549,7 +7666,7 @@
         <v>44</v>
       </c>
       <c r="H72" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I72" s="5"/>
       <c r="J72" s="5">
@@ -7579,7 +7696,7 @@
         <v>44</v>
       </c>
       <c r="H73" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I73" s="5"/>
       <c r="J73" s="5">
@@ -7609,7 +7726,7 @@
         <v>44</v>
       </c>
       <c r="H74" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I74" s="5"/>
       <c r="J74" s="5">
@@ -7639,7 +7756,7 @@
         <v>44</v>
       </c>
       <c r="H75" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I75" s="5"/>
       <c r="J75" s="5">
@@ -7654,7 +7771,7 @@
         <v>155</v>
       </c>
       <c r="C76" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D76" s="1">
         <v>400000000</v>
@@ -7669,7 +7786,7 @@
         <v>44</v>
       </c>
       <c r="H76" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I76" s="5"/>
       <c r="J76" s="5">
@@ -7699,7 +7816,7 @@
         <v>44</v>
       </c>
       <c r="H77" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I77" s="5"/>
       <c r="J77" s="5">
@@ -7729,7 +7846,7 @@
         <v>44</v>
       </c>
       <c r="H78" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I78" s="5"/>
       <c r="J78" s="5">
@@ -7744,7 +7861,7 @@
         <v>159</v>
       </c>
       <c r="C79" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D79" s="1">
         <v>1003724736</v>
@@ -7759,7 +7876,7 @@
         <v>44</v>
       </c>
       <c r="H79" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I79" s="5"/>
       <c r="J79" s="5">
@@ -7789,7 +7906,7 @@
         <v>44</v>
       </c>
       <c r="H80" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I80" s="5"/>
       <c r="J80" s="5">
@@ -7819,7 +7936,7 @@
         <v>44</v>
       </c>
       <c r="H81" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I81" s="5"/>
       <c r="J81" s="5">
@@ -7834,7 +7951,7 @@
         <v>161</v>
       </c>
       <c r="C82" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D82" s="1">
         <v>181124998</v>
@@ -7849,7 +7966,7 @@
         <v>44</v>
       </c>
       <c r="H82" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I82" s="5"/>
       <c r="J82" s="5"/>
@@ -7874,10 +7991,10 @@
         <v>308345333</v>
       </c>
       <c r="G83" t="s">
-        <v>106</v>
+        <v>92</v>
       </c>
       <c r="H83" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I83" s="5"/>
       <c r="J83" s="5">
@@ -7892,7 +8009,7 @@
         <v>162</v>
       </c>
       <c r="C84" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D84" s="1">
         <v>456179013</v>
@@ -7904,10 +8021,10 @@
         <v>464380516</v>
       </c>
       <c r="G84" t="s">
-        <v>106</v>
+        <v>92</v>
       </c>
       <c r="H84" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I84" s="5"/>
       <c r="J84" s="5">
@@ -7934,10 +8051,10 @@
         <v>367521178</v>
       </c>
       <c r="G85" t="s">
-        <v>106</v>
+        <v>92</v>
       </c>
       <c r="H85" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I85" s="5"/>
       <c r="J85" s="5">
@@ -7964,10 +8081,10 @@
         <v>412290581</v>
       </c>
       <c r="G86" t="s">
-        <v>106</v>
+        <v>92</v>
       </c>
       <c r="H86" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I86" s="5"/>
       <c r="J86" s="5">
@@ -7997,7 +8114,7 @@
         <v>44</v>
       </c>
       <c r="H87" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I87" s="5"/>
       <c r="J87" s="5">
@@ -8027,7 +8144,7 @@
         <v>44</v>
       </c>
       <c r="H88" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I88" s="5"/>
       <c r="J88" s="5">
@@ -8057,7 +8174,7 @@
         <v>44</v>
       </c>
       <c r="H89" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I89" s="5"/>
       <c r="J89" s="5">
@@ -8087,7 +8204,7 @@
         <v>44</v>
       </c>
       <c r="H90" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I90" s="5"/>
       <c r="J90" s="5">
@@ -8117,7 +8234,7 @@
         <v>44</v>
       </c>
       <c r="H91" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I91" s="5"/>
       <c r="J91" s="5">
@@ -8147,7 +8264,7 @@
         <v>44</v>
       </c>
       <c r="H92" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I92" s="5"/>
       <c r="J92" s="5"/>
@@ -8172,10 +8289,10 @@
         <v>275639320</v>
       </c>
       <c r="G93" t="s">
-        <v>106</v>
+        <v>92</v>
       </c>
       <c r="H93" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I93" s="5"/>
       <c r="J93" s="5"/>
@@ -8188,7 +8305,7 @@
         <v>170</v>
       </c>
       <c r="C94" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D94" s="1">
         <v>440558255</v>
@@ -8200,10 +8317,10 @@
         <v>442701115</v>
       </c>
       <c r="G94" t="s">
-        <v>106</v>
+        <v>92</v>
       </c>
       <c r="H94" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I94" s="5"/>
       <c r="J94" s="5"/>
@@ -8228,10 +8345,10 @@
         <v>446332480</v>
       </c>
       <c r="G95" t="s">
-        <v>106</v>
+        <v>92</v>
       </c>
       <c r="H95" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I95" s="5"/>
       <c r="J95" s="5"/>
@@ -8259,7 +8376,7 @@
         <v>44</v>
       </c>
       <c r="H96" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I96" s="5"/>
       <c r="J96" s="5">
@@ -8289,7 +8406,7 @@
         <v>44</v>
       </c>
       <c r="H97" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I97" s="5"/>
       <c r="J97" s="5">
@@ -8304,7 +8421,7 @@
         <v>127</v>
       </c>
       <c r="C98" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D98" s="1">
         <v>157982595</v>
@@ -8319,7 +8436,7 @@
         <v>44</v>
       </c>
       <c r="H98" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I98" s="5"/>
       <c r="J98" s="5">
@@ -8349,7 +8466,7 @@
         <v>44</v>
       </c>
       <c r="H99" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I99" s="5"/>
       <c r="J99" s="5">
@@ -8379,7 +8496,7 @@
         <v>44</v>
       </c>
       <c r="H100" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I100" s="5"/>
       <c r="J100" s="5"/>
@@ -8407,7 +8524,7 @@
         <v>44</v>
       </c>
       <c r="H101" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I101" s="5"/>
       <c r="J101" s="5"/>
@@ -8435,7 +8552,7 @@
         <v>44</v>
       </c>
       <c r="H102" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I102" s="5"/>
       <c r="J102" s="5"/>
@@ -8448,7 +8565,7 @@
         <v>172</v>
       </c>
       <c r="C103" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D103" s="1">
         <v>116977839</v>
@@ -8463,7 +8580,7 @@
         <v>44</v>
       </c>
       <c r="H103" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I103" s="5"/>
       <c r="J103" s="5"/>
@@ -8491,7 +8608,7 @@
         <v>44</v>
       </c>
       <c r="H104" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I104" s="5"/>
       <c r="J104" s="5"/>
@@ -8519,7 +8636,7 @@
         <v>44</v>
       </c>
       <c r="H105" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I105" s="5"/>
       <c r="J105" s="5"/>
@@ -8547,7 +8664,7 @@
         <v>44</v>
       </c>
       <c r="H106" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I106" s="5"/>
       <c r="J106" s="5">
@@ -8562,7 +8679,7 @@
         <v>139</v>
       </c>
       <c r="C107" t="s">
-        <v>173</v>
+        <v>141</v>
       </c>
       <c r="D107" s="1">
         <v>60000000</v>
@@ -8577,7 +8694,7 @@
         <v>44</v>
       </c>
       <c r="H107" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I107" s="5"/>
       <c r="J107" s="5">
@@ -8607,7 +8724,7 @@
         <v>44</v>
       </c>
       <c r="H108" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I108" s="5"/>
       <c r="J108" s="5">
@@ -8637,7 +8754,7 @@
         <v>44</v>
       </c>
       <c r="H109" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I109" s="5"/>
       <c r="J109" s="5">
@@ -8649,29 +8766,29 @@
         <v>7</v>
       </c>
       <c r="B110" t="s">
-        <v>68</v>
+        <v>173</v>
       </c>
       <c r="C110" t="s">
-        <v>60</v>
+        <v>114</v>
       </c>
       <c r="D110" s="1">
-        <v>500000000</v>
+        <v>946084601</v>
       </c>
       <c r="E110" s="1">
-        <v>1165423958</v>
+        <v>1255172172</v>
       </c>
       <c r="F110" s="7">
-        <v>-188251002</v>
+        <v>86029794</v>
       </c>
       <c r="G110" t="s">
         <v>44</v>
       </c>
       <c r="H110" t="s">
-        <v>45</v>
+        <v>96</v>
       </c>
       <c r="I110" s="5"/>
       <c r="J110" s="5">
-        <v>1.2554</v>
+        <v>0.6374</v>
       </c>
     </row>
     <row r="111" spans="1:10" x14ac:dyDescent="0.25">
@@ -8679,29 +8796,29 @@
         <v>7</v>
       </c>
       <c r="B111" t="s">
-        <v>68</v>
+        <v>174</v>
       </c>
       <c r="C111" t="s">
-        <v>48</v>
+        <v>97</v>
       </c>
       <c r="D111" s="1">
-        <v>500000000</v>
+        <v>274323144</v>
       </c>
       <c r="E111" s="1">
-        <v>1151125436</v>
+        <v>374599171</v>
       </c>
       <c r="F111" s="7">
-        <v>-183539197</v>
+        <v>-1221560</v>
       </c>
       <c r="G111" t="s">
         <v>44</v>
       </c>
       <c r="H111" t="s">
-        <v>45</v>
+        <v>96</v>
       </c>
       <c r="I111" s="5"/>
       <c r="J111" s="5">
-        <v>1.2554</v>
+        <v>0.36829999999999996</v>
       </c>
     </row>
     <row r="112" spans="1:10" x14ac:dyDescent="0.25">
@@ -8709,29 +8826,29 @@
         <v>7</v>
       </c>
       <c r="B112" t="s">
-        <v>68</v>
+        <v>175</v>
       </c>
       <c r="C112" t="s">
-        <v>43</v>
+        <v>115</v>
       </c>
       <c r="D112" s="1">
-        <v>500000000</v>
+        <v>314964360</v>
       </c>
       <c r="E112" s="1">
-        <v>1148829895</v>
+        <v>337505230</v>
       </c>
       <c r="F112" s="7">
-        <v>-208539973</v>
+        <v>-2653247</v>
       </c>
       <c r="G112" t="s">
         <v>44</v>
       </c>
       <c r="H112" t="s">
-        <v>45</v>
+        <v>96</v>
       </c>
       <c r="I112" s="5"/>
       <c r="J112" s="5">
-        <v>1.2554</v>
+        <v>0.0633</v>
       </c>
     </row>
     <row r="113" spans="1:10" x14ac:dyDescent="0.25">
@@ -8739,29 +8856,29 @@
         <v>7</v>
       </c>
       <c r="B113" t="s">
-        <v>68</v>
+        <v>175</v>
       </c>
       <c r="C113" t="s">
-        <v>50</v>
+        <v>99</v>
       </c>
       <c r="D113" s="1">
-        <v>500000000</v>
+        <v>1151650255</v>
       </c>
       <c r="E113" s="1">
-        <v>1186966069</v>
+        <v>1214682638</v>
       </c>
       <c r="F113" s="7">
-        <v>-204454782</v>
+        <v>-11725692</v>
       </c>
       <c r="G113" t="s">
         <v>44</v>
       </c>
       <c r="H113" t="s">
-        <v>45</v>
+        <v>96</v>
       </c>
       <c r="I113" s="5"/>
       <c r="J113" s="5">
-        <v>1.2554</v>
+        <v>0.0633</v>
       </c>
     </row>
     <row r="114" spans="1:10" x14ac:dyDescent="0.25">
@@ -8769,29 +8886,29 @@
         <v>7</v>
       </c>
       <c r="B114" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="C114" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="D114" s="1">
-        <v>946084601</v>
+        <v>823846300</v>
       </c>
       <c r="E114" s="1">
-        <v>1255172172</v>
+        <v>997557132</v>
       </c>
       <c r="F114" s="7">
-        <v>86029794</v>
+        <v>-18297135</v>
       </c>
       <c r="G114" t="s">
         <v>44</v>
       </c>
       <c r="H114" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I114" s="5"/>
       <c r="J114" s="5">
-        <v>0.6374</v>
+        <v>0.21989999999999998</v>
       </c>
     </row>
     <row r="115" spans="1:10" x14ac:dyDescent="0.25">
@@ -8799,29 +8916,29 @@
         <v>7</v>
       </c>
       <c r="B115" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C115" t="s">
-        <v>96</v>
+        <v>121</v>
       </c>
       <c r="D115" s="1">
-        <v>274323144</v>
+        <v>820369757</v>
       </c>
       <c r="E115" s="1">
-        <v>374599171</v>
+        <v>988168804</v>
       </c>
       <c r="F115" s="7">
-        <v>-1221560</v>
+        <v>-15019704</v>
       </c>
       <c r="G115" t="s">
         <v>44</v>
       </c>
       <c r="H115" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I115" s="5"/>
       <c r="J115" s="5">
-        <v>0.36829999999999996</v>
+        <v>0.21989999999999998</v>
       </c>
     </row>
     <row r="116" spans="1:10" x14ac:dyDescent="0.25">
@@ -8832,26 +8949,26 @@
         <v>176</v>
       </c>
       <c r="C116" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="D116" s="1">
-        <v>314964360</v>
+        <v>822731626</v>
       </c>
       <c r="E116" s="1">
-        <v>337505230</v>
+        <v>993985391</v>
       </c>
       <c r="F116" s="7">
-        <v>-2653247</v>
+        <v>-17743111</v>
       </c>
       <c r="G116" t="s">
         <v>44</v>
       </c>
       <c r="H116" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I116" s="5"/>
       <c r="J116" s="5">
-        <v>0.0633</v>
+        <v>0.21989999999999998</v>
       </c>
     </row>
     <row r="117" spans="1:10" x14ac:dyDescent="0.25">
@@ -8859,29 +8976,29 @@
         <v>7</v>
       </c>
       <c r="B117" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C117" t="s">
-        <v>98</v>
+        <v>135</v>
       </c>
       <c r="D117" s="1">
-        <v>1151650255</v>
+        <v>425389351</v>
       </c>
       <c r="E117" s="1">
-        <v>1214682638</v>
+        <v>475239009</v>
       </c>
       <c r="F117" s="7">
-        <v>-11725692</v>
+        <v>9432028</v>
       </c>
       <c r="G117" t="s">
         <v>44</v>
       </c>
       <c r="H117" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I117" s="5"/>
       <c r="J117" s="5">
-        <v>0.0633</v>
+        <v>0.1247</v>
       </c>
     </row>
     <row r="118" spans="1:10" x14ac:dyDescent="0.25">
@@ -8892,26 +9009,26 @@
         <v>177</v>
       </c>
       <c r="C118" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="D118" s="1">
-        <v>823846300</v>
+        <v>508571279</v>
       </c>
       <c r="E118" s="1">
-        <v>997557132</v>
+        <v>578473784</v>
       </c>
       <c r="F118" s="7">
-        <v>-18297135</v>
+        <v>1973545</v>
       </c>
       <c r="G118" t="s">
         <v>44</v>
       </c>
       <c r="H118" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I118" s="5"/>
       <c r="J118" s="5">
-        <v>0.21989999999999998</v>
+        <v>0.1247</v>
       </c>
     </row>
     <row r="119" spans="1:10" x14ac:dyDescent="0.25">
@@ -8922,26 +9039,26 @@
         <v>177</v>
       </c>
       <c r="C119" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="D119" s="1">
-        <v>820369757</v>
+        <v>464478952</v>
       </c>
       <c r="E119" s="1">
-        <v>988168804</v>
+        <v>511250642</v>
       </c>
       <c r="F119" s="7">
-        <v>-15019704</v>
+        <v>-186646</v>
       </c>
       <c r="G119" t="s">
         <v>44</v>
       </c>
       <c r="H119" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I119" s="5"/>
       <c r="J119" s="5">
-        <v>0.21989999999999998</v>
+        <v>0.1247</v>
       </c>
     </row>
     <row r="120" spans="1:10" x14ac:dyDescent="0.25">
@@ -8949,29 +9066,29 @@
         <v>7</v>
       </c>
       <c r="B120" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C120" t="s">
-        <v>122</v>
+        <v>140</v>
       </c>
       <c r="D120" s="1">
-        <v>822731626</v>
+        <v>627191291</v>
       </c>
       <c r="E120" s="1">
-        <v>993985391</v>
+        <v>714504487</v>
       </c>
       <c r="F120" s="7">
-        <v>-17743111</v>
+        <v>18107712</v>
       </c>
       <c r="G120" t="s">
         <v>44</v>
       </c>
       <c r="H120" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I120" s="5"/>
       <c r="J120" s="5">
-        <v>0.21989999999999998</v>
+        <v>0.1307</v>
       </c>
     </row>
     <row r="121" spans="1:10" x14ac:dyDescent="0.25">
@@ -8982,26 +9099,26 @@
         <v>178</v>
       </c>
       <c r="C121" t="s">
-        <v>135</v>
+        <v>179</v>
       </c>
       <c r="D121" s="1">
-        <v>425389351</v>
+        <v>425091462</v>
       </c>
       <c r="E121" s="1">
-        <v>475239009</v>
+        <v>478192278</v>
       </c>
       <c r="F121" s="7">
-        <v>9432028</v>
+        <v>10642444</v>
       </c>
       <c r="G121" t="s">
         <v>44</v>
       </c>
       <c r="H121" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I121" s="5"/>
       <c r="J121" s="5">
-        <v>0.1247</v>
+        <v>0.1307</v>
       </c>
     </row>
     <row r="122" spans="1:10" x14ac:dyDescent="0.25">
@@ -9009,89 +9126,85 @@
         <v>7</v>
       </c>
       <c r="B122" t="s">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="C122" t="s">
-        <v>124</v>
+        <v>101</v>
       </c>
       <c r="D122" s="1">
-        <v>508571279</v>
+        <v>428950000</v>
       </c>
       <c r="E122" s="1">
-        <v>578473784</v>
+        <v>431428553</v>
       </c>
       <c r="F122" s="7">
-        <v>1973545</v>
+        <v>431428553</v>
       </c>
       <c r="G122" t="s">
-        <v>44</v>
+        <v>92</v>
       </c>
       <c r="H122" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I122" s="5"/>
-      <c r="J122" s="5">
-        <v>0.1247</v>
-      </c>
+      <c r="J122" s="5"/>
     </row>
     <row r="123" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>7</v>
       </c>
       <c r="B123" t="s">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="C123" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="D123" s="1">
-        <v>464478952</v>
+        <v>462463907</v>
       </c>
       <c r="E123" s="1">
-        <v>511250642</v>
+        <v>466146222</v>
       </c>
       <c r="F123" s="7">
-        <v>-186646</v>
+        <v>466146222</v>
       </c>
       <c r="G123" t="s">
-        <v>44</v>
+        <v>92</v>
       </c>
       <c r="H123" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I123" s="5"/>
-      <c r="J123" s="5">
-        <v>0.1247</v>
-      </c>
+      <c r="J123" s="5"/>
     </row>
     <row r="124" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>7</v>
       </c>
       <c r="B124" t="s">
-        <v>179</v>
+        <v>126</v>
       </c>
       <c r="C124" t="s">
-        <v>140</v>
+        <v>79</v>
       </c>
       <c r="D124" s="1">
-        <v>627191291</v>
+        <v>151969815</v>
       </c>
       <c r="E124" s="1">
-        <v>714504487</v>
+        <v>266710574</v>
       </c>
       <c r="F124" s="7">
-        <v>18107712</v>
+        <v>-10002997</v>
       </c>
       <c r="G124" t="s">
         <v>44</v>
       </c>
       <c r="H124" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I124" s="5"/>
       <c r="J124" s="5">
-        <v>0.1307</v>
+        <v>0.6866</v>
       </c>
     </row>
     <row r="125" spans="1:10" x14ac:dyDescent="0.25">
@@ -9099,55 +9212,53 @@
         <v>7</v>
       </c>
       <c r="B125" t="s">
-        <v>179</v>
+        <v>129</v>
       </c>
       <c r="C125" t="s">
-        <v>180</v>
+        <v>130</v>
       </c>
       <c r="D125" s="1">
-        <v>425091462</v>
+        <v>105992843</v>
       </c>
       <c r="E125" s="1">
-        <v>478192278</v>
+        <v>129828838</v>
       </c>
       <c r="F125" s="7">
-        <v>10642444</v>
+        <v>127284</v>
       </c>
       <c r="G125" t="s">
         <v>44</v>
       </c>
       <c r="H125" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I125" s="5"/>
-      <c r="J125" s="5">
-        <v>0.1307</v>
-      </c>
+      <c r="J125" s="5"/>
     </row>
     <row r="126" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>7</v>
       </c>
       <c r="B126" t="s">
-        <v>170</v>
+        <v>129</v>
       </c>
       <c r="C126" t="s">
-        <v>100</v>
+        <v>131</v>
       </c>
       <c r="D126" s="1">
-        <v>428950000</v>
+        <v>258094745</v>
       </c>
       <c r="E126" s="1">
-        <v>431428553</v>
+        <v>333870078</v>
       </c>
       <c r="F126" s="7">
-        <v>431428553</v>
+        <v>649752</v>
       </c>
       <c r="G126" t="s">
-        <v>106</v>
+        <v>44</v>
       </c>
       <c r="H126" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I126" s="5"/>
       <c r="J126" s="5"/>
@@ -9157,171 +9268,177 @@
         <v>7</v>
       </c>
       <c r="B127" t="s">
-        <v>170</v>
+        <v>129</v>
       </c>
       <c r="C127" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="D127" s="1">
-        <v>462463907</v>
+        <v>299312934</v>
       </c>
       <c r="E127" s="1">
-        <v>466146222</v>
+        <v>373139760</v>
       </c>
       <c r="F127" s="7">
-        <v>466146222</v>
+        <v>61623</v>
       </c>
       <c r="G127" t="s">
-        <v>106</v>
+        <v>44</v>
       </c>
       <c r="H127" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I127" s="5"/>
       <c r="J127" s="5"/>
     </row>
     <row r="128" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B128" t="s">
-        <v>126</v>
+        <v>176</v>
       </c>
       <c r="C128" t="s">
-        <v>79</v>
+        <v>120</v>
       </c>
       <c r="D128" s="1">
-        <v>151969815</v>
+        <v>510820499</v>
       </c>
       <c r="E128" s="1">
-        <v>266710574</v>
+        <v>619202327</v>
       </c>
       <c r="F128" s="7">
-        <v>-10002997</v>
+        <v>-11343656</v>
       </c>
       <c r="G128" t="s">
         <v>44</v>
       </c>
       <c r="H128" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I128" s="5"/>
       <c r="J128" s="5">
-        <v>0.6866</v>
+        <v>0.21989999999999998</v>
       </c>
     </row>
     <row r="129" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B129" t="s">
-        <v>129</v>
+        <v>176</v>
       </c>
       <c r="C129" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
       <c r="D129" s="1">
-        <v>105992843</v>
+        <v>508402028</v>
       </c>
       <c r="E129" s="1">
-        <v>129828838</v>
+        <v>612836264</v>
       </c>
       <c r="F129" s="7">
-        <v>127284</v>
+        <v>-9349078</v>
       </c>
       <c r="G129" t="s">
         <v>44</v>
       </c>
       <c r="H129" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I129" s="5"/>
-      <c r="J129" s="5"/>
+      <c r="J129" s="5">
+        <v>0.21989999999999998</v>
+      </c>
     </row>
     <row r="130" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B130" t="s">
-        <v>129</v>
+        <v>178</v>
       </c>
       <c r="C130" t="s">
-        <v>131</v>
+        <v>140</v>
       </c>
       <c r="D130" s="1">
-        <v>258094745</v>
+        <v>378735074</v>
       </c>
       <c r="E130" s="1">
-        <v>333870078</v>
+        <v>430909955</v>
       </c>
       <c r="F130" s="7">
-        <v>649752</v>
+        <v>10920693</v>
       </c>
       <c r="G130" t="s">
         <v>44</v>
       </c>
       <c r="H130" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I130" s="5"/>
-      <c r="J130" s="5"/>
+      <c r="J130" s="5">
+        <v>0.1307</v>
+      </c>
     </row>
     <row r="131" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B131" t="s">
-        <v>129</v>
+        <v>178</v>
       </c>
       <c r="C131" t="s">
-        <v>132</v>
+        <v>118</v>
       </c>
       <c r="D131" s="1">
-        <v>299312934</v>
+        <v>339081835</v>
       </c>
       <c r="E131" s="1">
-        <v>373139760</v>
+        <v>334549088</v>
       </c>
       <c r="F131" s="7">
-        <v>61623</v>
+        <v>334549088</v>
       </c>
       <c r="G131" t="s">
-        <v>44</v>
+        <v>92</v>
       </c>
       <c r="H131" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I131" s="5"/>
-      <c r="J131" s="5"/>
+      <c r="J131" s="5">
+        <v>-0.0173</v>
+      </c>
     </row>
     <row r="132" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>8</v>
       </c>
       <c r="B132" t="s">
-        <v>177</v>
+        <v>126</v>
       </c>
       <c r="C132" t="s">
-        <v>120</v>
+        <v>79</v>
       </c>
       <c r="D132" s="1">
-        <v>510820499</v>
+        <v>151227051</v>
       </c>
       <c r="E132" s="1">
-        <v>619202327</v>
+        <v>265114862</v>
       </c>
       <c r="F132" s="7">
-        <v>-11343656</v>
+        <v>-9882162</v>
       </c>
       <c r="G132" t="s">
         <v>44</v>
       </c>
       <c r="H132" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I132" s="5"/>
       <c r="J132" s="5">
-        <v>0.21989999999999998</v>
+        <v>0.6866</v>
       </c>
     </row>
     <row r="133" spans="1:10" x14ac:dyDescent="0.25">
@@ -9329,29 +9446,29 @@
         <v>8</v>
       </c>
       <c r="B133" t="s">
-        <v>177</v>
+        <v>127</v>
       </c>
       <c r="C133" t="s">
-        <v>121</v>
+        <v>79</v>
       </c>
       <c r="D133" s="1">
-        <v>508402028</v>
+        <v>159277445</v>
       </c>
       <c r="E133" s="1">
-        <v>612836264</v>
+        <v>304979599</v>
       </c>
       <c r="F133" s="7">
-        <v>-9349078</v>
+        <v>-1188805</v>
       </c>
       <c r="G133" t="s">
         <v>44</v>
       </c>
       <c r="H133" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I133" s="5"/>
       <c r="J133" s="5">
-        <v>0.21989999999999998</v>
+        <v>0.914</v>
       </c>
     </row>
     <row r="134" spans="1:10" x14ac:dyDescent="0.25">
@@ -9359,29 +9476,29 @@
         <v>8</v>
       </c>
       <c r="B134" t="s">
-        <v>179</v>
+        <v>127</v>
       </c>
       <c r="C134" t="s">
-        <v>140</v>
+        <v>128</v>
       </c>
       <c r="D134" s="1">
-        <v>378735074</v>
+        <v>159101214</v>
       </c>
       <c r="E134" s="1">
-        <v>430909955</v>
+        <v>311496128</v>
       </c>
       <c r="F134" s="7">
-        <v>10920693</v>
+        <v>-330845</v>
       </c>
       <c r="G134" t="s">
         <v>44</v>
       </c>
       <c r="H134" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I134" s="5"/>
       <c r="J134" s="5">
-        <v>0.1307</v>
+        <v>0.914</v>
       </c>
     </row>
     <row r="135" spans="1:10" x14ac:dyDescent="0.25">
@@ -9389,29 +9506,29 @@
         <v>8</v>
       </c>
       <c r="B135" t="s">
-        <v>179</v>
+        <v>127</v>
       </c>
       <c r="C135" t="s">
-        <v>118</v>
+        <v>105</v>
       </c>
       <c r="D135" s="1">
-        <v>339081835</v>
+        <v>159382615</v>
       </c>
       <c r="E135" s="1">
-        <v>334549088</v>
+        <v>311580226</v>
       </c>
       <c r="F135" s="7">
-        <v>334549088</v>
+        <v>-493569</v>
       </c>
       <c r="G135" t="s">
-        <v>106</v>
+        <v>44</v>
       </c>
       <c r="H135" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I135" s="5"/>
       <c r="J135" s="5">
-        <v>-0.0173</v>
+        <v>0.914</v>
       </c>
     </row>
     <row r="136" spans="1:10" x14ac:dyDescent="0.25">
@@ -9419,29 +9536,29 @@
         <v>8</v>
       </c>
       <c r="B136" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C136" t="s">
-        <v>79</v>
+        <v>120</v>
       </c>
       <c r="D136" s="1">
-        <v>151227051</v>
+        <v>159708987</v>
       </c>
       <c r="E136" s="1">
-        <v>265114862</v>
+        <v>309819784</v>
       </c>
       <c r="F136" s="7">
-        <v>-9882162</v>
+        <v>-813461</v>
       </c>
       <c r="G136" t="s">
         <v>44</v>
       </c>
       <c r="H136" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I136" s="5"/>
       <c r="J136" s="5">
-        <v>0.6866</v>
+        <v>0.914</v>
       </c>
     </row>
     <row r="137" spans="1:10" x14ac:dyDescent="0.25">
@@ -9449,145 +9566,137 @@
         <v>8</v>
       </c>
       <c r="B137" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C137" t="s">
-        <v>79</v>
+        <v>130</v>
       </c>
       <c r="D137" s="1">
-        <v>159277445</v>
+        <v>106848757</v>
       </c>
       <c r="E137" s="1">
-        <v>304979599</v>
+        <v>130862848</v>
       </c>
       <c r="F137" s="7">
-        <v>-1188805</v>
+        <v>124527</v>
       </c>
       <c r="G137" t="s">
         <v>44</v>
       </c>
       <c r="H137" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I137" s="5"/>
-      <c r="J137" s="5">
-        <v>0.914</v>
-      </c>
+      <c r="J137" s="5"/>
     </row>
     <row r="138" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>8</v>
       </c>
       <c r="B138" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C138" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="D138" s="1">
-        <v>159101214</v>
+        <v>134102607</v>
       </c>
       <c r="E138" s="1">
-        <v>311496128</v>
+        <v>174702263</v>
       </c>
       <c r="F138" s="7">
-        <v>-330845</v>
+        <v>342198</v>
       </c>
       <c r="G138" t="s">
         <v>44</v>
       </c>
       <c r="H138" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I138" s="5"/>
-      <c r="J138" s="5">
-        <v>0.914</v>
-      </c>
+      <c r="J138" s="5"/>
     </row>
     <row r="139" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>8</v>
       </c>
       <c r="B139" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C139" t="s">
-        <v>104</v>
+        <v>132</v>
       </c>
       <c r="D139" s="1">
-        <v>159382615</v>
+        <v>257027478</v>
       </c>
       <c r="E139" s="1">
-        <v>311580226</v>
+        <v>319545179</v>
       </c>
       <c r="F139" s="7">
-        <v>-493569</v>
+        <v>142366</v>
       </c>
       <c r="G139" t="s">
         <v>44</v>
       </c>
       <c r="H139" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I139" s="5"/>
-      <c r="J139" s="5">
-        <v>0.914</v>
-      </c>
+      <c r="J139" s="5"/>
     </row>
     <row r="140" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>8</v>
       </c>
       <c r="B140" t="s">
-        <v>127</v>
+        <v>172</v>
       </c>
       <c r="C140" t="s">
-        <v>120</v>
+        <v>103</v>
       </c>
       <c r="D140" s="1">
-        <v>159708987</v>
+        <v>160873068</v>
       </c>
       <c r="E140" s="1">
-        <v>309819784</v>
+        <v>257650149</v>
       </c>
       <c r="F140" s="7">
-        <v>-813461</v>
+        <v>4148152</v>
       </c>
       <c r="G140" t="s">
         <v>44</v>
       </c>
       <c r="H140" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I140" s="5"/>
-      <c r="J140" s="5">
-        <v>0.914</v>
-      </c>
+      <c r="J140" s="5"/>
     </row>
     <row r="141" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>8</v>
       </c>
       <c r="B141" t="s">
-        <v>129</v>
+        <v>172</v>
       </c>
       <c r="C141" t="s">
-        <v>130</v>
+        <v>115</v>
       </c>
       <c r="D141" s="1">
-        <v>106848757</v>
+        <v>163472383</v>
       </c>
       <c r="E141" s="1">
-        <v>130862848</v>
+        <v>221410107</v>
       </c>
       <c r="F141" s="7">
-        <v>124527</v>
+        <v>1745193</v>
       </c>
       <c r="G141" t="s">
         <v>44</v>
       </c>
       <c r="H141" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I141" s="5"/>
       <c r="J141" s="5"/>
@@ -9597,25 +9706,25 @@
         <v>8</v>
       </c>
       <c r="B142" t="s">
-        <v>129</v>
+        <v>172</v>
       </c>
       <c r="C142" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="D142" s="1">
-        <v>134102607</v>
+        <v>161120051</v>
       </c>
       <c r="E142" s="1">
-        <v>174702263</v>
+        <v>234838962</v>
       </c>
       <c r="F142" s="7">
-        <v>342198</v>
+        <v>1796960</v>
       </c>
       <c r="G142" t="s">
         <v>44</v>
       </c>
       <c r="H142" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I142" s="5"/>
       <c r="J142" s="5"/>
@@ -9625,25 +9734,25 @@
         <v>8</v>
       </c>
       <c r="B143" t="s">
-        <v>129</v>
+        <v>172</v>
       </c>
       <c r="C143" t="s">
-        <v>132</v>
+        <v>105</v>
       </c>
       <c r="D143" s="1">
-        <v>257027478</v>
+        <v>149737366</v>
       </c>
       <c r="E143" s="1">
-        <v>319545179</v>
+        <v>220527203</v>
       </c>
       <c r="F143" s="7">
-        <v>142366</v>
+        <v>10349727</v>
       </c>
       <c r="G143" t="s">
         <v>44</v>
       </c>
       <c r="H143" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I143" s="5"/>
       <c r="J143" s="5"/>
@@ -9653,109 +9762,115 @@
         <v>8</v>
       </c>
       <c r="B144" t="s">
-        <v>172</v>
+        <v>137</v>
       </c>
       <c r="C144" t="s">
-        <v>102</v>
+        <v>138</v>
       </c>
       <c r="D144" s="1">
-        <v>160873068</v>
+        <v>170770415</v>
       </c>
       <c r="E144" s="1">
-        <v>257650149</v>
+        <v>169160821</v>
       </c>
       <c r="F144" s="7">
-        <v>4148152</v>
+        <v>-2713085</v>
       </c>
       <c r="G144" t="s">
         <v>44</v>
       </c>
       <c r="H144" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I144" s="5"/>
-      <c r="J144" s="5"/>
+      <c r="J144" s="5">
+        <v>-0.0070999999999999995</v>
+      </c>
     </row>
     <row r="145" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>8</v>
       </c>
       <c r="B145" t="s">
-        <v>172</v>
+        <v>137</v>
       </c>
       <c r="C145" t="s">
-        <v>115</v>
+        <v>101</v>
       </c>
       <c r="D145" s="1">
-        <v>163472383</v>
+        <v>92866928</v>
       </c>
       <c r="E145" s="1">
-        <v>221410107</v>
+        <v>92150680</v>
       </c>
       <c r="F145" s="7">
-        <v>1745193</v>
+        <v>-1474945</v>
       </c>
       <c r="G145" t="s">
         <v>44</v>
       </c>
       <c r="H145" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I145" s="5"/>
-      <c r="J145" s="5"/>
+      <c r="J145" s="5">
+        <v>-0.0070999999999999995</v>
+      </c>
     </row>
     <row r="146" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
         <v>8</v>
       </c>
       <c r="B146" t="s">
-        <v>172</v>
+        <v>137</v>
       </c>
       <c r="C146" t="s">
-        <v>134</v>
+        <v>99</v>
       </c>
       <c r="D146" s="1">
-        <v>161120051</v>
+        <v>116515080</v>
       </c>
       <c r="E146" s="1">
-        <v>234838962</v>
+        <v>115478381</v>
       </c>
       <c r="F146" s="7">
-        <v>1796960</v>
+        <v>-1835166</v>
       </c>
       <c r="G146" t="s">
         <v>44</v>
       </c>
       <c r="H146" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I146" s="5"/>
-      <c r="J146" s="5"/>
+      <c r="J146" s="5">
+        <v>-0.0070999999999999995</v>
+      </c>
     </row>
     <row r="147" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>8</v>
       </c>
       <c r="B147" t="s">
-        <v>172</v>
+        <v>142</v>
       </c>
       <c r="C147" t="s">
-        <v>104</v>
+        <v>131</v>
       </c>
       <c r="D147" s="1">
-        <v>149737366</v>
+        <v>60000000</v>
       </c>
       <c r="E147" s="1">
-        <v>220527203</v>
+        <v>76839686</v>
       </c>
       <c r="F147" s="7">
-        <v>10349727</v>
+        <v>-2121898</v>
       </c>
       <c r="G147" t="s">
         <v>44</v>
       </c>
       <c r="H147" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I147" s="5"/>
       <c r="J147" s="5"/>
@@ -9765,90 +9880,84 @@
         <v>8</v>
       </c>
       <c r="B148" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="C148" t="s">
-        <v>138</v>
+        <v>101</v>
       </c>
       <c r="D148" s="1">
-        <v>170770415</v>
+        <v>60000000</v>
       </c>
       <c r="E148" s="1">
-        <v>169160821</v>
+        <v>72935938</v>
       </c>
       <c r="F148" s="7">
-        <v>-2713085</v>
+        <v>-73692729</v>
       </c>
       <c r="G148" t="s">
         <v>44</v>
       </c>
       <c r="H148" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I148" s="5"/>
-      <c r="J148" s="5">
-        <v>-0.0070999999999999995</v>
-      </c>
+      <c r="J148" s="5"/>
     </row>
     <row r="149" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
         <v>8</v>
       </c>
       <c r="B149" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="C149" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D149" s="1">
-        <v>92866928</v>
+        <v>120000000</v>
       </c>
       <c r="E149" s="1">
-        <v>92150680</v>
+        <v>146792233</v>
       </c>
       <c r="F149" s="7">
-        <v>-1474945</v>
+        <v>163566</v>
       </c>
       <c r="G149" t="s">
         <v>44</v>
       </c>
       <c r="H149" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I149" s="5"/>
-      <c r="J149" s="5">
-        <v>-0.0070999999999999995</v>
-      </c>
+      <c r="J149" s="5"/>
     </row>
     <row r="150" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>8</v>
       </c>
       <c r="B150" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="C150" t="s">
-        <v>98</v>
+        <v>144</v>
       </c>
       <c r="D150" s="1">
-        <v>116515080</v>
+        <v>100000000</v>
       </c>
       <c r="E150" s="1">
-        <v>115478381</v>
+        <v>133483168</v>
       </c>
       <c r="F150" s="7">
-        <v>-1835166</v>
+        <v>-25400</v>
       </c>
       <c r="G150" t="s">
         <v>44</v>
       </c>
       <c r="H150" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I150" s="5"/>
-      <c r="J150" s="5">
-        <v>-0.0070999999999999995</v>
-      </c>
+      <c r="J150" s="5"/>
     </row>
     <row r="151" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
@@ -9858,22 +9967,22 @@
         <v>142</v>
       </c>
       <c r="C151" t="s">
-        <v>131</v>
+        <v>145</v>
       </c>
       <c r="D151" s="1">
         <v>60000000</v>
       </c>
       <c r="E151" s="1">
-        <v>76839686</v>
+        <v>75654265</v>
       </c>
       <c r="F151" s="7">
-        <v>-2121898</v>
+        <v>-485923</v>
       </c>
       <c r="G151" t="s">
         <v>44</v>
       </c>
       <c r="H151" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I151" s="5"/>
       <c r="J151" s="5"/>
@@ -9883,137 +9992,145 @@
         <v>8</v>
       </c>
       <c r="B152" t="s">
-        <v>142</v>
+        <v>180</v>
       </c>
       <c r="C152" t="s">
-        <v>100</v>
+        <v>59</v>
       </c>
       <c r="D152" s="1">
         <v>60000000</v>
       </c>
       <c r="E152" s="1">
-        <v>72935938</v>
+        <v>89122293</v>
       </c>
       <c r="F152" s="7">
-        <v>-73692729</v>
+        <v>-1236575</v>
       </c>
       <c r="G152" t="s">
         <v>44</v>
       </c>
       <c r="H152" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I152" s="5"/>
-      <c r="J152" s="5"/>
+      <c r="J152" s="5">
+        <v>0.7315</v>
+      </c>
     </row>
     <row r="153" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
         <v>8</v>
       </c>
       <c r="B153" t="s">
-        <v>142</v>
+        <v>180</v>
       </c>
       <c r="C153" t="s">
-        <v>100</v>
+        <v>121</v>
       </c>
       <c r="D153" s="1">
-        <v>120000000</v>
+        <v>60000000</v>
       </c>
       <c r="E153" s="1">
-        <v>146792233</v>
+        <v>85570319</v>
       </c>
       <c r="F153" s="7">
-        <v>163566</v>
+        <v>-950764</v>
       </c>
       <c r="G153" t="s">
         <v>44</v>
       </c>
       <c r="H153" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I153" s="5"/>
-      <c r="J153" s="5"/>
+      <c r="J153" s="5">
+        <v>0.7315</v>
+      </c>
     </row>
     <row r="154" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
         <v>8</v>
       </c>
       <c r="B154" t="s">
-        <v>142</v>
+        <v>180</v>
       </c>
       <c r="C154" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="D154" s="1">
-        <v>100000000</v>
+        <v>60000000</v>
       </c>
       <c r="E154" s="1">
-        <v>133483168</v>
+        <v>87308547</v>
       </c>
       <c r="F154" s="7">
-        <v>-25400</v>
+        <v>-471520</v>
       </c>
       <c r="G154" t="s">
         <v>44</v>
       </c>
       <c r="H154" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I154" s="5"/>
-      <c r="J154" s="5"/>
+      <c r="J154" s="5">
+        <v>0.7315</v>
+      </c>
     </row>
     <row r="155" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
         <v>8</v>
       </c>
       <c r="B155" t="s">
-        <v>142</v>
+        <v>180</v>
       </c>
       <c r="C155" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D155" s="1">
         <v>60000000</v>
       </c>
       <c r="E155" s="1">
-        <v>75654265</v>
+        <v>84636837</v>
       </c>
       <c r="F155" s="7">
-        <v>-485923</v>
+        <v>241555</v>
       </c>
       <c r="G155" t="s">
         <v>44</v>
       </c>
       <c r="H155" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I155" s="5"/>
-      <c r="J155" s="5"/>
+      <c r="J155" s="5">
+        <v>0.7315</v>
+      </c>
     </row>
     <row r="156" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
         <v>8</v>
       </c>
       <c r="B156" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C156" t="s">
-        <v>59</v>
+        <v>115</v>
       </c>
       <c r="D156" s="1">
         <v>60000000</v>
       </c>
       <c r="E156" s="1">
-        <v>89122293</v>
+        <v>88954199</v>
       </c>
       <c r="F156" s="7">
-        <v>-1236575</v>
+        <v>-817882</v>
       </c>
       <c r="G156" t="s">
         <v>44</v>
       </c>
       <c r="H156" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I156" s="5"/>
       <c r="J156" s="5">
@@ -10025,29 +10142,29 @@
         <v>8</v>
       </c>
       <c r="B157" t="s">
-        <v>181</v>
+        <v>151</v>
       </c>
       <c r="C157" t="s">
-        <v>121</v>
+        <v>152</v>
       </c>
       <c r="D157" s="1">
-        <v>60000000</v>
+        <v>100000000</v>
       </c>
       <c r="E157" s="1">
-        <v>85570319</v>
+        <v>134048105</v>
       </c>
       <c r="F157" s="7">
-        <v>-950764</v>
+        <v>-178481</v>
       </c>
       <c r="G157" t="s">
         <v>44</v>
       </c>
       <c r="H157" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I157" s="5"/>
       <c r="J157" s="5">
-        <v>0.7315</v>
+        <v>0.4351</v>
       </c>
     </row>
     <row r="158" spans="1:10" x14ac:dyDescent="0.25">
@@ -10055,29 +10172,29 @@
         <v>8</v>
       </c>
       <c r="B158" t="s">
-        <v>181</v>
+        <v>151</v>
       </c>
       <c r="C158" t="s">
-        <v>148</v>
+        <v>121</v>
       </c>
       <c r="D158" s="1">
-        <v>60000000</v>
+        <v>100000000</v>
       </c>
       <c r="E158" s="1">
-        <v>87308547</v>
+        <v>136597280</v>
       </c>
       <c r="F158" s="7">
-        <v>-471520</v>
+        <v>54421</v>
       </c>
       <c r="G158" t="s">
         <v>44</v>
       </c>
       <c r="H158" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I158" s="5"/>
       <c r="J158" s="5">
-        <v>0.7315</v>
+        <v>0.4351</v>
       </c>
     </row>
     <row r="159" spans="1:10" x14ac:dyDescent="0.25">
@@ -10085,29 +10202,29 @@
         <v>8</v>
       </c>
       <c r="B159" t="s">
-        <v>181</v>
+        <v>151</v>
       </c>
       <c r="C159" t="s">
-        <v>144</v>
+        <v>105</v>
       </c>
       <c r="D159" s="1">
-        <v>60000000</v>
+        <v>100000000</v>
       </c>
       <c r="E159" s="1">
-        <v>84636837</v>
+        <v>137179366</v>
       </c>
       <c r="F159" s="7">
-        <v>241555</v>
+        <v>333074</v>
       </c>
       <c r="G159" t="s">
         <v>44</v>
       </c>
       <c r="H159" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I159" s="5"/>
       <c r="J159" s="5">
-        <v>0.7315</v>
+        <v>0.4351</v>
       </c>
     </row>
     <row r="160" spans="1:10" x14ac:dyDescent="0.25">
@@ -10115,150 +10232,142 @@
         <v>8</v>
       </c>
       <c r="B160" t="s">
-        <v>181</v>
+        <v>151</v>
       </c>
       <c r="C160" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="D160" s="1">
-        <v>60000000</v>
+        <v>100000000</v>
       </c>
       <c r="E160" s="1">
-        <v>88954199</v>
+        <v>136973911</v>
       </c>
       <c r="F160" s="7">
-        <v>-817882</v>
+        <v>235488</v>
       </c>
       <c r="G160" t="s">
         <v>44</v>
       </c>
       <c r="H160" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I160" s="5"/>
       <c r="J160" s="5">
-        <v>0.7315</v>
+        <v>0.4351</v>
       </c>
     </row>
     <row r="161" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="B161" t="s">
-        <v>151</v>
+        <v>181</v>
       </c>
       <c r="C161" t="s">
-        <v>152</v>
+        <v>105</v>
       </c>
       <c r="D161" s="1">
-        <v>100000000</v>
+        <v>0</v>
       </c>
       <c r="E161" s="1">
-        <v>134048105</v>
+        <v>0</v>
       </c>
       <c r="F161" s="7">
-        <v>-178481</v>
+        <v>-1683240295</v>
       </c>
       <c r="G161" t="s">
-        <v>44</v>
+        <v>93</v>
       </c>
       <c r="H161" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I161" s="5"/>
-      <c r="J161" s="5">
-        <v>0.4351</v>
-      </c>
+      <c r="J161" s="5"/>
     </row>
     <row r="162" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="B162" t="s">
-        <v>151</v>
+        <v>181</v>
       </c>
       <c r="C162" t="s">
-        <v>121</v>
+        <v>79</v>
       </c>
       <c r="D162" s="1">
-        <v>100000000</v>
+        <v>0</v>
       </c>
       <c r="E162" s="1">
-        <v>136597280</v>
+        <v>0</v>
       </c>
       <c r="F162" s="7">
-        <v>54421</v>
+        <v>-1687228552</v>
       </c>
       <c r="G162" t="s">
-        <v>44</v>
+        <v>93</v>
       </c>
       <c r="H162" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I162" s="5"/>
-      <c r="J162" s="5">
-        <v>0.4351</v>
-      </c>
+      <c r="J162" s="5"/>
     </row>
     <row r="163" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="B163" t="s">
-        <v>151</v>
+        <v>119</v>
       </c>
       <c r="C163" t="s">
-        <v>104</v>
+        <v>147</v>
       </c>
       <c r="D163" s="1">
-        <v>100000000</v>
+        <v>0</v>
       </c>
       <c r="E163" s="1">
-        <v>137179366</v>
+        <v>0</v>
       </c>
       <c r="F163" s="7">
-        <v>333074</v>
+        <v>-3924793719</v>
       </c>
       <c r="G163" t="s">
-        <v>44</v>
+        <v>93</v>
       </c>
       <c r="H163" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I163" s="5"/>
-      <c r="J163" s="5">
-        <v>0.4351</v>
-      </c>
+      <c r="J163" s="5"/>
     </row>
     <row r="164" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="B164" t="s">
-        <v>151</v>
+        <v>182</v>
       </c>
       <c r="C164" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="D164" s="1">
-        <v>100000000</v>
+        <v>0</v>
       </c>
       <c r="E164" s="1">
-        <v>136973911</v>
+        <v>0</v>
       </c>
       <c r="F164" s="7">
-        <v>235488</v>
+        <v>-1314198402</v>
       </c>
       <c r="G164" t="s">
-        <v>44</v>
+        <v>93</v>
       </c>
       <c r="H164" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I164" s="5"/>
-      <c r="J164" s="5">
-        <v>0.4351</v>
-      </c>
+      <c r="J164" s="5"/>
     </row>
     <row r="165" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
@@ -10268,7 +10377,7 @@
         <v>182</v>
       </c>
       <c r="C165" t="s">
-        <v>104</v>
+        <v>125</v>
       </c>
       <c r="D165" s="1">
         <v>0</v>
@@ -10277,13 +10386,13 @@
         <v>0</v>
       </c>
       <c r="F165" s="7">
-        <v>-1683240295</v>
+        <v>-1837050463</v>
       </c>
       <c r="G165" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H165" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I165" s="5"/>
       <c r="J165" s="5"/>
@@ -10293,10 +10402,10 @@
         <v>5</v>
       </c>
       <c r="B166" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C166" t="s">
-        <v>79</v>
+        <v>171</v>
       </c>
       <c r="D166" s="1">
         <v>0</v>
@@ -10305,13 +10414,13 @@
         <v>0</v>
       </c>
       <c r="F166" s="7">
-        <v>-1687228552</v>
+        <v>-1216881012</v>
       </c>
       <c r="G166" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H166" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I166" s="5"/>
       <c r="J166" s="5"/>
@@ -10321,10 +10430,10 @@
         <v>5</v>
       </c>
       <c r="B167" t="s">
-        <v>119</v>
+        <v>183</v>
       </c>
       <c r="C167" t="s">
-        <v>147</v>
+        <v>101</v>
       </c>
       <c r="D167" s="1">
         <v>0</v>
@@ -10333,13 +10442,13 @@
         <v>0</v>
       </c>
       <c r="F167" s="7">
-        <v>-3924793719</v>
+        <v>-2051054273</v>
       </c>
       <c r="G167" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H167" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I167" s="5"/>
       <c r="J167" s="5"/>
@@ -10352,7 +10461,7 @@
         <v>183</v>
       </c>
       <c r="C168" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="D168" s="1">
         <v>0</v>
@@ -10361,13 +10470,13 @@
         <v>0</v>
       </c>
       <c r="F168" s="7">
-        <v>-1314198402</v>
+        <v>-1508632702</v>
       </c>
       <c r="G168" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H168" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I168" s="5"/>
       <c r="J168" s="5"/>
@@ -10380,7 +10489,7 @@
         <v>183</v>
       </c>
       <c r="C169" t="s">
-        <v>125</v>
+        <v>184</v>
       </c>
       <c r="D169" s="1">
         <v>0</v>
@@ -10389,13 +10498,13 @@
         <v>0</v>
       </c>
       <c r="F169" s="7">
-        <v>-1837050463</v>
+        <v>-422609458</v>
       </c>
       <c r="G169" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H169" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I169" s="5"/>
       <c r="J169" s="5"/>
@@ -10405,10 +10514,10 @@
         <v>5</v>
       </c>
       <c r="B170" t="s">
-        <v>184</v>
+        <v>151</v>
       </c>
       <c r="C170" t="s">
-        <v>171</v>
+        <v>147</v>
       </c>
       <c r="D170" s="1">
         <v>0</v>
@@ -10417,26 +10526,26 @@
         <v>0</v>
       </c>
       <c r="F170" s="7">
-        <v>-1216881012</v>
+        <v>-543970609</v>
       </c>
       <c r="G170" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H170" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I170" s="5"/>
       <c r="J170" s="5"/>
     </row>
     <row r="171" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B171" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C171" t="s">
-        <v>100</v>
+        <v>79</v>
       </c>
       <c r="D171" s="1">
         <v>0</v>
@@ -10445,26 +10554,26 @@
         <v>0</v>
       </c>
       <c r="F171" s="7">
-        <v>-2051054273</v>
+        <v>-303753501</v>
       </c>
       <c r="G171" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H171" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I171" s="5"/>
       <c r="J171" s="5"/>
     </row>
     <row r="172" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B172" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C172" t="s">
-        <v>128</v>
+        <v>105</v>
       </c>
       <c r="D172" s="1">
         <v>0</v>
@@ -10473,26 +10582,26 @@
         <v>0</v>
       </c>
       <c r="F172" s="7">
-        <v>-1508632702</v>
+        <v>-456179013</v>
       </c>
       <c r="G172" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H172" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I172" s="5"/>
       <c r="J172" s="5"/>
     </row>
     <row r="173" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B173" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C173" t="s">
-        <v>185</v>
+        <v>163</v>
       </c>
       <c r="D173" s="1">
         <v>0</v>
@@ -10501,26 +10610,26 @@
         <v>0</v>
       </c>
       <c r="F173" s="7">
-        <v>-422609458</v>
+        <v>-361201485</v>
       </c>
       <c r="G173" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H173" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I173" s="5"/>
       <c r="J173" s="5"/>
     </row>
     <row r="174" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B174" t="s">
-        <v>151</v>
+        <v>185</v>
       </c>
       <c r="C174" t="s">
-        <v>147</v>
+        <v>135</v>
       </c>
       <c r="D174" s="1">
         <v>0</v>
@@ -10529,13 +10638,13 @@
         <v>0</v>
       </c>
       <c r="F174" s="7">
-        <v>-543970609</v>
+        <v>-405779245</v>
       </c>
       <c r="G174" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H174" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I174" s="5"/>
       <c r="J174" s="5"/>
@@ -10545,10 +10654,10 @@
         <v>6</v>
       </c>
       <c r="B175" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="C175" t="s">
-        <v>79</v>
+        <v>171</v>
       </c>
       <c r="D175" s="1">
         <v>0</v>
@@ -10557,13 +10666,13 @@
         <v>0</v>
       </c>
       <c r="F175" s="7">
-        <v>-303753501</v>
+        <v>-282822171</v>
       </c>
       <c r="G175" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H175" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I175" s="5"/>
       <c r="J175" s="5"/>
@@ -10573,10 +10682,10 @@
         <v>6</v>
       </c>
       <c r="B176" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="C176" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D176" s="1">
         <v>0</v>
@@ -10585,13 +10694,13 @@
         <v>0</v>
       </c>
       <c r="F176" s="7">
-        <v>-456179013</v>
+        <v>-746373228</v>
       </c>
       <c r="G176" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H176" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I176" s="5"/>
       <c r="J176" s="5"/>
@@ -10601,10 +10710,10 @@
         <v>6</v>
       </c>
       <c r="B177" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="C177" t="s">
-        <v>163</v>
+        <v>128</v>
       </c>
       <c r="D177" s="1">
         <v>0</v>
@@ -10613,13 +10722,13 @@
         <v>0</v>
       </c>
       <c r="F177" s="7">
-        <v>-361201485</v>
+        <v>-442398214</v>
       </c>
       <c r="G177" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H177" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I177" s="5"/>
       <c r="J177" s="5"/>
@@ -10629,10 +10738,10 @@
         <v>6</v>
       </c>
       <c r="B178" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="C178" t="s">
-        <v>135</v>
+        <v>184</v>
       </c>
       <c r="D178" s="1">
         <v>0</v>
@@ -10641,26 +10750,26 @@
         <v>0</v>
       </c>
       <c r="F178" s="7">
-        <v>-405779245</v>
+        <v>-216266708</v>
       </c>
       <c r="G178" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H178" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I178" s="5"/>
       <c r="J178" s="5"/>
     </row>
     <row r="179" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B179" t="s">
-        <v>184</v>
+        <v>68</v>
       </c>
       <c r="C179" t="s">
-        <v>171</v>
+        <v>60</v>
       </c>
       <c r="D179" s="1">
         <v>0</v>
@@ -10669,26 +10778,26 @@
         <v>0</v>
       </c>
       <c r="F179" s="7">
-        <v>-282822171</v>
+        <v>-1353674960</v>
       </c>
       <c r="G179" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H179" t="s">
-        <v>95</v>
+        <v>45</v>
       </c>
       <c r="I179" s="5"/>
       <c r="J179" s="5"/>
     </row>
     <row r="180" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B180" t="s">
-        <v>184</v>
+        <v>68</v>
       </c>
       <c r="C180" t="s">
-        <v>100</v>
+        <v>48</v>
       </c>
       <c r="D180" s="1">
         <v>0</v>
@@ -10697,26 +10806,26 @@
         <v>0</v>
       </c>
       <c r="F180" s="7">
-        <v>-746373228</v>
+        <v>-1334664633</v>
       </c>
       <c r="G180" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H180" t="s">
-        <v>95</v>
+        <v>45</v>
       </c>
       <c r="I180" s="5"/>
       <c r="J180" s="5"/>
     </row>
     <row r="181" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B181" t="s">
-        <v>184</v>
+        <v>68</v>
       </c>
       <c r="C181" t="s">
-        <v>128</v>
+        <v>43</v>
       </c>
       <c r="D181" s="1">
         <v>0</v>
@@ -10725,26 +10834,26 @@
         <v>0</v>
       </c>
       <c r="F181" s="7">
-        <v>-442398214</v>
+        <v>-1357369868</v>
       </c>
       <c r="G181" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H181" t="s">
-        <v>95</v>
+        <v>45</v>
       </c>
       <c r="I181" s="5"/>
       <c r="J181" s="5"/>
     </row>
     <row r="182" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B182" t="s">
-        <v>184</v>
+        <v>68</v>
       </c>
       <c r="C182" t="s">
-        <v>185</v>
+        <v>50</v>
       </c>
       <c r="D182" s="1">
         <v>0</v>
@@ -10753,13 +10862,13 @@
         <v>0</v>
       </c>
       <c r="F182" s="7">
-        <v>-216266708</v>
+        <v>-1391420851</v>
       </c>
       <c r="G182" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H182" t="s">
-        <v>95</v>
+        <v>45</v>
       </c>
       <c r="I182" s="5"/>
       <c r="J182" s="5"/>
@@ -10769,10 +10878,10 @@
         <v>7</v>
       </c>
       <c r="B183" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C183" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D183" s="1">
         <v>0</v>
@@ -10784,10 +10893,10 @@
         <v>-534717371</v>
       </c>
       <c r="G183" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H183" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I183" s="5"/>
       <c r="J183" s="5"/>
@@ -10797,7 +10906,7 @@
         <v>7</v>
       </c>
       <c r="B184" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C184" t="s">
         <v>128</v>
@@ -10812,10 +10921,10 @@
         <v>-461631869</v>
       </c>
       <c r="G184" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H184" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I184" s="5"/>
       <c r="J184" s="5"/>
@@ -10825,7 +10934,7 @@
         <v>8</v>
       </c>
       <c r="B185" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C185" t="s">
         <v>118</v>
@@ -10840,10 +10949,10 @@
         <v>-333967279</v>
       </c>
       <c r="G185" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H185" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I185" s="5"/>
       <c r="J185" s="5"/>
@@ -10868,10 +10977,10 @@
         <v>-73420942</v>
       </c>
       <c r="G186" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H186" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I186" s="5"/>
       <c r="J186" s="5"/>

</xml_diff>